<commit_message>
Update median of 4 clusters (factoriescap_s (costs) 0).xlsx
</commit_message>
<xml_diff>
--- a/clustering/median of 4 clusters (factoriescap_s (costs) 0).xlsx
+++ b/clustering/median of 4 clusters (factoriescap_s (costs) 0).xlsx
@@ -1,37 +1,72 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Albert\.spyder-py3\ITMO-3\clustering\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="5">
+  <si>
+    <t>clust</t>
+  </si>
+  <si>
+    <t>factoriescap_s</t>
+  </si>
+  <si>
+    <t>ITcosts_s</t>
+  </si>
+  <si>
+    <t>skvozcosts_s</t>
+  </si>
+  <si>
+    <t>trainingcosts_s</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000%"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +81,51 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Процентный" xfId="1" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,110 +413,296 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>clust</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>factoriescap_s</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>ITcosts_s</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>skvozcosts_s</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>trainingcosts_s</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="n">
-        <v>1783343.499999995</v>
-      </c>
-      <c r="C2" t="n">
-        <v>4252.421610759988</v>
-      </c>
-      <c r="D2" t="n">
-        <v>13.5522009199999</v>
-      </c>
-      <c r="E2" t="n">
-        <v>6.340581079999491</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="n">
-        <v>13968260.99999999</v>
-      </c>
-      <c r="C3" t="n">
-        <v>38168.40288759999</v>
-      </c>
-      <c r="D3" t="n">
-        <v>5240.677482</v>
-      </c>
-      <c r="E3" t="n">
-        <v>11.97612415999989</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="n">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1783343.4999999951</v>
+      </c>
+      <c r="C2" s="2">
+        <v>4252.4216107599877</v>
+      </c>
+      <c r="D2" s="2">
+        <v>13.552200919999899</v>
+      </c>
+      <c r="E2" s="2">
+        <v>6.3405810799994908</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <v>13968260.999999991</v>
+      </c>
+      <c r="C3" s="2">
+        <v>38168.402887599987</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5240.6774820000001</v>
+      </c>
+      <c r="E3" s="2">
+        <v>11.976124159999889</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
         <v>64887516</v>
       </c>
-      <c r="C4" t="n">
-        <v>227928.64269201</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1518.59722925</v>
-      </c>
-      <c r="E4" t="n">
-        <v>877.1140827399996</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="C4" s="2">
+        <v>227928.64269201001</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1518.5972292500001</v>
+      </c>
+      <c r="E4" s="2">
+        <v>877.11408273999962</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" t="n">
-        <v>12161153.99999999</v>
-      </c>
-      <c r="C5" t="n">
-        <v>35568.66195351</v>
-      </c>
-      <c r="D5" t="n">
-        <v>592.1307466199997</v>
-      </c>
-      <c r="E5" t="n">
-        <v>6413.502227579999</v>
+      <c r="B5" s="2">
+        <v>12161153.999999991</v>
+      </c>
+      <c r="C5" s="2">
+        <v>35568.661953510004</v>
+      </c>
+      <c r="D5" s="2">
+        <v>592.13074661999974</v>
+      </c>
+      <c r="E5" s="2">
+        <v>6413.5022275799993</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>0</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1783343.4999999951</v>
+      </c>
+      <c r="C9" s="3">
+        <f>C2/$B2</f>
+        <v>2.384521888665868E-3</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" ref="D9:E9" si="0">D2/$B2</f>
+        <v>7.5993216786333853E-6</v>
+      </c>
+      <c r="E9" s="3">
+        <f t="shared" si="0"/>
+        <v>3.5554457568042881E-6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2">
+        <v>13968260.999999991</v>
+      </c>
+      <c r="C10" s="3">
+        <f t="shared" ref="C10:E10" si="1">C3/$B3</f>
+        <v>2.732509285701349E-3</v>
+      </c>
+      <c r="D10" s="3">
+        <f t="shared" si="1"/>
+        <v>3.7518467631725977E-4</v>
+      </c>
+      <c r="E10" s="3">
+        <f t="shared" si="1"/>
+        <v>8.5738118438651011E-7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>2</v>
+      </c>
+      <c r="B11" s="2">
+        <v>64887516</v>
+      </c>
+      <c r="C11" s="3">
+        <f t="shared" ref="C11:E11" si="2">C4/$B4</f>
+        <v>3.5126732651009481E-3</v>
+      </c>
+      <c r="D11" s="3">
+        <f t="shared" si="2"/>
+        <v>2.3403534652952349E-5</v>
+      </c>
+      <c r="E11" s="3">
+        <f t="shared" si="2"/>
+        <v>1.3517455079340679E-5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>3</v>
+      </c>
+      <c r="B12" s="2">
+        <v>12161153.999999991</v>
+      </c>
+      <c r="C12" s="3">
+        <f t="shared" ref="C12:E12" si="3">C5/$B5</f>
+        <v>2.9247768717927617E-3</v>
+      </c>
+      <c r="D12" s="3">
+        <f t="shared" si="3"/>
+        <v>4.8690341937944393E-5</v>
+      </c>
+      <c r="E12" s="3">
+        <f t="shared" si="3"/>
+        <v>5.273761213434189E-4</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B5">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C5">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D5">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E5">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9:B12">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:C12">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9:D12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9:E12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>